<commit_message>
Update mobile_transactions.xlsx with new transaction data
</commit_message>
<xml_diff>
--- a/datasets/raw/mobile_transactions.xlsx
+++ b/datasets/raw/mobile_transactions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\wifi-or-data-anaytics\datasets\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9957F285-B836-43F4-9A68-A6332439BA19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10F870CE-3719-42C7-93F0-1E02E9E79C8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{2245BC4D-441C-49AF-98C4-92169C979341}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="8">
   <si>
     <t>date</t>
   </si>
@@ -59,7 +59,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="170" formatCode="yyyy/mm/dd"/>
+    <numFmt numFmtId="164" formatCode="yyyy/mm/dd"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -93,7 +93,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1014,22 +1014,39 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" s="1"/>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="2">
+        <v>46317</v>
+      </c>
+      <c r="B33" t="s">
+        <v>6</v>
+      </c>
+      <c r="C33">
+        <v>25000</v>
+      </c>
+      <c r="D33">
+        <v>14</v>
+      </c>
+      <c r="E33">
+        <v>7</v>
+      </c>
+      <c r="F33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="1"/>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="1"/>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="1"/>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="1"/>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="1"/>
     </row>
   </sheetData>

</xml_diff>